<commit_message>
Fix pontaj Excel consolidated export details
</commit_message>
<xml_diff>
--- a/public/templates/pontaj-consolidat-template.xlsx
+++ b/public/templates/pontaj-consolidat-template.xlsx
@@ -7917,9 +7917,7 @@
       <c r="E59" s="166">
         <v>2</v>
       </c>
-      <c r="F59" s="529" t="s">
-        <v>50</v>
-      </c>
+      <c r="F59" s="529"/>
       <c r="G59" s="529"/>
       <c r="H59" s="529"/>
       <c r="I59" s="529"/>
@@ -29822,9 +29820,7 @@
       <c r="E59" s="166">
         <v>2</v>
       </c>
-      <c r="F59" s="529" t="s">
-        <v>186</v>
-      </c>
+      <c r="F59" s="529"/>
       <c r="G59" s="529"/>
       <c r="H59" s="529"/>
       <c r="I59" s="529"/>
@@ -36886,9 +36882,7 @@
       <c r="C59" s="164"/>
       <c r="D59" s="451"/>
       <c r="E59" s="166"/>
-      <c r="F59" s="529" t="s">
-        <v>5</v>
-      </c>
+      <c r="F59" s="529"/>
       <c r="G59" s="529"/>
       <c r="H59" s="529"/>
       <c r="I59" s="529"/>

</xml_diff>